<commit_message>
update with waste management
</commit_message>
<xml_diff>
--- a/projects/WasteCGE/data/wasteDataMapping.xlsx
+++ b/projects/WasteCGE/data/wasteDataMapping.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxj477\Documents\GitHub\CGE_Generator\projects\WasteCGE\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F6443E-2778-40D5-B6F3-00BCB3DDC6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42A632A-CEA8-442C-89DF-5CFAD78853F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03ECE533-816B-43DE-A89C-B52A0D8DBA42}"/>
   </bookViews>
   <sheets>
     <sheet name="s" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="182">
   <si>
     <t>010000</t>
   </si>
@@ -570,6 +570,18 @@
   </si>
   <si>
     <t>off</t>
+  </si>
+  <si>
+    <t>sGRS</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Waste</t>
   </si>
 </sst>
 </file>
@@ -1332,13 +1344,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD5B5ABD-6DF9-4822-82B4-672ADF465860}">
-  <dimension ref="A1:C147"/>
+  <dimension ref="A1:D147"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>176</v>
       </c>
@@ -1348,8 +1360,11 @@
       <c r="C1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A2" s="71" t="s">
         <v>137</v>
       </c>
@@ -1359,8 +1374,11 @@
       <c r="C2" s="24" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A3" s="71" t="s">
         <v>138</v>
       </c>
@@ -1368,8 +1386,11 @@
       <c r="C3" s="24" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A4" s="71" t="s">
         <v>139</v>
       </c>
@@ -1377,8 +1398,11 @@
       <c r="C4" s="24" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A5" s="71" t="s">
         <v>140</v>
       </c>
@@ -1386,8 +1410,11 @@
       <c r="C5" s="24" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A6" s="71" t="s">
         <v>141</v>
       </c>
@@ -1395,8 +1422,11 @@
       <c r="C6" s="24" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A7" s="71" t="s">
         <v>142</v>
       </c>
@@ -1404,8 +1434,11 @@
       <c r="C7" s="24" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A8" s="71" t="s">
         <v>143</v>
       </c>
@@ -1413,8 +1446,11 @@
       <c r="C8" s="24" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A9" s="71" t="s">
         <v>144</v>
       </c>
@@ -1422,8 +1458,11 @@
       <c r="C9" s="24" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A10" s="71" t="s">
         <v>145</v>
       </c>
@@ -1431,8 +1470,11 @@
       <c r="C10" s="24" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="71" t="s">
         <v>146</v>
       </c>
@@ -1440,8 +1482,11 @@
       <c r="C11" s="24" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A12" s="71" t="s">
         <v>147</v>
       </c>
@@ -1449,8 +1494,11 @@
       <c r="C12" s="24" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A13" s="71" t="s">
         <v>148</v>
       </c>
@@ -1458,8 +1506,11 @@
       <c r="C13" s="24" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D13" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A14" s="71" t="s">
         <v>149</v>
       </c>
@@ -1467,8 +1518,11 @@
       <c r="C14" s="25" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A15" s="71" t="s">
         <v>1</v>
       </c>
@@ -1478,8 +1532,11 @@
       <c r="C15" s="26" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D15" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A16" s="71" t="s">
         <v>2</v>
       </c>
@@ -1489,8 +1546,11 @@
       <c r="C16" s="27" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D16" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A17" s="72" t="s">
         <v>3</v>
       </c>
@@ -1500,8 +1560,11 @@
       <c r="C17" s="28" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D17" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A18" s="71" t="s">
         <v>4</v>
       </c>
@@ -1509,8 +1572,11 @@
         <v>4</v>
       </c>
       <c r="C18" s="29"/>
-    </row>
-    <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D18" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A19" s="71" t="s">
         <v>5</v>
       </c>
@@ -1518,8 +1584,11 @@
         <v>5</v>
       </c>
       <c r="C19" s="30"/>
-    </row>
-    <row r="20" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D19" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A20" s="71" t="s">
         <v>6</v>
       </c>
@@ -1529,8 +1598,11 @@
       <c r="C20" s="31">
         <v>10011</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D20" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A21" s="71" t="s">
         <v>7</v>
       </c>
@@ -1540,8 +1612,11 @@
       <c r="C21" s="32">
         <v>10020</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D21" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A22" s="71" t="s">
         <v>8</v>
       </c>
@@ -1551,8 +1626,11 @@
       <c r="C22" s="32">
         <v>10030</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D22" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A23" s="71" t="s">
         <v>9</v>
       </c>
@@ -1562,8 +1640,11 @@
       <c r="C23" s="32">
         <v>10040</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D23" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A24" s="71" t="s">
         <v>10</v>
       </c>
@@ -1573,8 +1654,11 @@
       <c r="C24" s="33">
         <v>10120</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A25" s="71" t="s">
         <v>11</v>
       </c>
@@ -1582,8 +1666,11 @@
         <v>11</v>
       </c>
       <c r="C25" s="34"/>
-    </row>
-    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D25" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A26" s="71" t="s">
         <v>12</v>
       </c>
@@ -1591,8 +1678,11 @@
         <v>12</v>
       </c>
       <c r="C26" s="35"/>
-    </row>
-    <row r="27" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A27" s="71" t="s">
         <v>13</v>
       </c>
@@ -1602,8 +1692,11 @@
       <c r="C27" s="36">
         <v>13150</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D27" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A28" s="71" t="s">
         <v>14</v>
       </c>
@@ -1611,8 +1704,11 @@
         <v>14</v>
       </c>
       <c r="C28" s="37"/>
-    </row>
-    <row r="29" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D28" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A29" s="71" t="s">
         <v>15</v>
       </c>
@@ -1620,8 +1716,11 @@
         <v>15</v>
       </c>
       <c r="C29" s="37"/>
-    </row>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D29" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A30" s="71" t="s">
         <v>16</v>
       </c>
@@ -1631,8 +1730,11 @@
       <c r="C30" s="32">
         <v>16000</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D30" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A31" s="71" t="s">
         <v>17</v>
       </c>
@@ -1642,8 +1744,11 @@
       <c r="C31" s="36">
         <v>25000</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D31" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A32" s="71" t="s">
         <v>18</v>
       </c>
@@ -1651,8 +1756,11 @@
         <v>18</v>
       </c>
       <c r="C32" s="37"/>
-    </row>
-    <row r="33" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D32" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A33" s="71" t="s">
         <v>19</v>
       </c>
@@ -1662,8 +1770,11 @@
       <c r="C33" s="38">
         <v>19000</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D33" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A34" s="71" t="s">
         <v>20</v>
       </c>
@@ -1673,8 +1784,11 @@
       <c r="C34" s="39">
         <v>20000</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D34" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A35" s="71" t="s">
         <v>21</v>
       </c>
@@ -1682,8 +1796,11 @@
         <v>21</v>
       </c>
       <c r="C35" s="40"/>
-    </row>
-    <row r="36" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D35" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A36" s="71" t="s">
         <v>22</v>
       </c>
@@ -1693,8 +1810,11 @@
       <c r="C36" s="41">
         <v>21000</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D36" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A37" s="71" t="s">
         <v>23</v>
       </c>
@@ -1704,8 +1824,11 @@
       <c r="C37" s="37">
         <v>25000</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D37" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A38" s="71" t="s">
         <v>24</v>
       </c>
@@ -1715,8 +1838,11 @@
       <c r="C38" s="42">
         <v>23001</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D38" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A39" s="71" t="s">
         <v>25</v>
       </c>
@@ -1726,8 +1852,11 @@
       <c r="C39" s="40">
         <v>23002</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D39" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A40" s="71" t="s">
         <v>26</v>
       </c>
@@ -1737,8 +1866,11 @@
       <c r="C40" s="37">
         <v>25000</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D40" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A41" s="71" t="s">
         <v>27</v>
       </c>
@@ -1746,8 +1878,11 @@
         <v>27</v>
       </c>
       <c r="C41" s="40"/>
-    </row>
-    <row r="42" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D41" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A42" s="71" t="s">
         <v>28</v>
       </c>
@@ -1757,8 +1892,11 @@
       <c r="C42" s="37">
         <v>13150</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D42" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A43" s="71" t="s">
         <v>29</v>
       </c>
@@ -1766,8 +1904,11 @@
         <v>29</v>
       </c>
       <c r="C43" s="37"/>
-    </row>
-    <row r="44" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D43" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A44" s="71" t="s">
         <v>30</v>
       </c>
@@ -1775,8 +1916,11 @@
         <v>30</v>
       </c>
       <c r="C44" s="37"/>
-    </row>
-    <row r="45" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D44" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A45" s="71" t="s">
         <v>31</v>
       </c>
@@ -1784,8 +1928,11 @@
         <v>31</v>
       </c>
       <c r="C45" s="37"/>
-    </row>
-    <row r="46" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D45" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A46" s="71" t="s">
         <v>32</v>
       </c>
@@ -1793,8 +1940,11 @@
         <v>32</v>
       </c>
       <c r="C46" s="37"/>
-    </row>
-    <row r="47" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D46" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A47" s="71" t="s">
         <v>33</v>
       </c>
@@ -1802,8 +1952,11 @@
         <v>33</v>
       </c>
       <c r="C47" s="37"/>
-    </row>
-    <row r="48" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D47" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A48" s="71" t="s">
         <v>34</v>
       </c>
@@ -1811,8 +1964,11 @@
         <v>34</v>
       </c>
       <c r="C48" s="37"/>
-    </row>
-    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D48" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A49" s="71" t="s">
         <v>35</v>
       </c>
@@ -1820,8 +1976,11 @@
         <v>35</v>
       </c>
       <c r="C49" s="37"/>
-    </row>
-    <row r="50" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D49" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A50" s="71" t="s">
         <v>36</v>
       </c>
@@ -1829,8 +1988,11 @@
         <v>36</v>
       </c>
       <c r="C50" s="37"/>
-    </row>
-    <row r="51" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D50" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A51" s="71" t="s">
         <v>37</v>
       </c>
@@ -1838,8 +2000,11 @@
         <v>37</v>
       </c>
       <c r="C51" s="37"/>
-    </row>
-    <row r="52" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D51" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A52" s="71" t="s">
         <v>38</v>
       </c>
@@ -1847,8 +2012,11 @@
         <v>38</v>
       </c>
       <c r="C52" s="37"/>
-    </row>
-    <row r="53" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D52" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A53" s="71" t="s">
         <v>39</v>
       </c>
@@ -1856,8 +2024,11 @@
         <v>39</v>
       </c>
       <c r="C53" s="40"/>
-    </row>
-    <row r="54" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D53" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A54" s="71" t="s">
         <v>40</v>
       </c>
@@ -1867,8 +2038,11 @@
       <c r="C54" s="37">
         <v>25000</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D54" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A55" s="73" t="s">
         <v>150</v>
       </c>
@@ -1878,15 +2052,21 @@
       <c r="C55" s="43" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D55" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A56" s="71" t="s">
         <v>151</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="44"/>
-    </row>
-    <row r="57" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D56" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A57" s="71" t="s">
         <v>42</v>
       </c>
@@ -1896,8 +2076,11 @@
       <c r="C57" s="45">
         <v>35002</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D57" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A58" s="71" t="s">
         <v>43</v>
       </c>
@@ -1907,8 +2090,11 @@
       <c r="C58" s="40">
         <v>35011</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D58" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A59" s="71" t="s">
         <v>44</v>
       </c>
@@ -1918,8 +2104,11 @@
       <c r="C59" s="46" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D59" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A60" s="71" t="s">
         <v>45</v>
       </c>
@@ -1929,8 +2118,11 @@
       <c r="C60" s="46" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D60" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A61" s="71" t="s">
         <v>152</v>
       </c>
@@ -1940,8 +2132,11 @@
       <c r="C61" s="76">
         <v>38391</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="D61" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A62" s="74" t="s">
         <v>153</v>
       </c>
@@ -1951,8 +2146,11 @@
       <c r="C62" s="76">
         <v>38392</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D62" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A63" s="71" t="s">
         <v>154</v>
       </c>
@@ -1962,8 +2160,11 @@
       <c r="C63" s="76">
         <v>38393</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D63" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A64" s="71" t="s">
         <v>155</v>
       </c>
@@ -1973,8 +2174,11 @@
       <c r="C64" s="76">
         <v>38392</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="D64" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A65" s="73" t="s">
         <v>156</v>
       </c>
@@ -1984,8 +2188,11 @@
       <c r="C65" s="76">
         <v>38392</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D65" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A66" s="74" t="s">
         <v>46</v>
       </c>
@@ -1995,8 +2202,11 @@
       <c r="C66" s="47" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D66" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A67" s="74" t="s">
         <v>47</v>
       </c>
@@ -2004,8 +2214,11 @@
         <v>47</v>
       </c>
       <c r="C67" s="48"/>
-    </row>
-    <row r="68" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D67" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A68" s="74" t="s">
         <v>48</v>
       </c>
@@ -2013,8 +2226,11 @@
         <v>48</v>
       </c>
       <c r="C68" s="49"/>
-    </row>
-    <row r="69" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D68" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A69" s="74" t="s">
         <v>49</v>
       </c>
@@ -2022,8 +2238,11 @@
         <v>49</v>
       </c>
       <c r="C69" s="50"/>
-    </row>
-    <row r="70" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D69" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A70" s="74" t="s">
         <v>50</v>
       </c>
@@ -2033,8 +2252,11 @@
       <c r="C70" s="51">
         <v>45000</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D70" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A71" s="74" t="s">
         <v>51</v>
       </c>
@@ -2042,8 +2264,11 @@
         <v>51</v>
       </c>
       <c r="C71" s="35"/>
-    </row>
-    <row r="72" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D71" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A72" s="74" t="s">
         <v>52</v>
       </c>
@@ -2053,8 +2278,11 @@
       <c r="C72" s="41">
         <v>46000</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D72" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A73" s="71" t="s">
         <v>53</v>
       </c>
@@ -2064,8 +2292,11 @@
       <c r="C73" s="52">
         <v>47000</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D73" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A74" s="71" t="s">
         <v>157</v>
       </c>
@@ -2075,8 +2306,11 @@
       <c r="C74" s="53">
         <v>49011</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D74" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A75" s="75" t="s">
         <v>158</v>
       </c>
@@ -2084,8 +2318,11 @@
       <c r="C75" s="53">
         <v>49011</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D75" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A76" s="71" t="s">
         <v>159</v>
       </c>
@@ -2095,8 +2332,11 @@
       <c r="C76" s="53">
         <v>49011</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D76" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A77" s="71" t="s">
         <v>160</v>
       </c>
@@ -2104,15 +2344,21 @@
       <c r="C77" s="54">
         <v>49024</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D77" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A78" s="71" t="s">
         <v>161</v>
       </c>
       <c r="B78" s="17"/>
       <c r="C78" s="55"/>
-    </row>
-    <row r="79" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D78" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A79" s="71" t="s">
         <v>162</v>
       </c>
@@ -2120,8 +2366,11 @@
       <c r="C79" s="54">
         <v>49024</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D79" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A80" s="73" t="s">
         <v>163</v>
       </c>
@@ -2131,15 +2380,21 @@
       <c r="C80" s="54">
         <v>49031</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D80" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A81" s="73" t="s">
         <v>164</v>
       </c>
       <c r="B81" s="18"/>
       <c r="C81" s="57"/>
-    </row>
-    <row r="82" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D81" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A82" s="73" t="s">
         <v>165</v>
       </c>
@@ -2147,8 +2402,11 @@
       <c r="C82" s="58">
         <v>49509</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D82" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A83" s="73" t="s">
         <v>166</v>
       </c>
@@ -2158,15 +2416,21 @@
       <c r="C83" s="59">
         <v>50001</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D83" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A84" s="73" t="s">
         <v>167</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="55"/>
-    </row>
-    <row r="85" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D84" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A85" s="73" t="s">
         <v>168</v>
       </c>
@@ -2174,8 +2438,11 @@
       <c r="C85" s="56">
         <v>49509</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D85" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A86" s="71" t="s">
         <v>169</v>
       </c>
@@ -2185,15 +2452,21 @@
       <c r="C86" s="60">
         <v>51001</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D86" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A87" s="71" t="s">
         <v>170</v>
       </c>
       <c r="B87" s="16"/>
       <c r="C87" s="61"/>
-    </row>
-    <row r="88" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D87" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A88" s="71" t="s">
         <v>171</v>
       </c>
@@ -2201,8 +2474,11 @@
       <c r="C88" s="62">
         <v>51009</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D88" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A89" s="71" t="s">
         <v>172</v>
       </c>
@@ -2212,15 +2488,21 @@
       <c r="C89" s="76">
         <v>53000</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D89" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A90" s="71" t="s">
         <v>173</v>
       </c>
       <c r="B90" s="21"/>
       <c r="C90" s="63"/>
-    </row>
-    <row r="91" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D90" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A91" s="71" t="s">
         <v>174</v>
       </c>
@@ -2230,15 +2512,21 @@
       <c r="C91" s="64" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D91" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A92" s="71" t="s">
         <v>175</v>
       </c>
       <c r="B92" s="12"/>
       <c r="C92" s="65"/>
-    </row>
-    <row r="93" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D92" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A93" s="71" t="s">
         <v>61</v>
       </c>
@@ -2248,8 +2536,11 @@
       <c r="C93" s="66">
         <v>55560</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D93" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A94" s="71" t="s">
         <v>62</v>
       </c>
@@ -2257,8 +2548,11 @@
         <v>62</v>
       </c>
       <c r="C94" s="66"/>
-    </row>
-    <row r="95" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D94" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A95" s="71" t="s">
         <v>63</v>
       </c>
@@ -2266,8 +2560,11 @@
         <v>63</v>
       </c>
       <c r="C95" s="66"/>
-    </row>
-    <row r="96" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D95" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A96" s="71" t="s">
         <v>64</v>
       </c>
@@ -2275,8 +2572,11 @@
         <v>64</v>
       </c>
       <c r="C96" s="66"/>
-    </row>
-    <row r="97" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D96" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A97" s="71" t="s">
         <v>65</v>
       </c>
@@ -2284,8 +2584,11 @@
         <v>65</v>
       </c>
       <c r="C97" s="66"/>
-    </row>
-    <row r="98" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D97" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A98" s="71" t="s">
         <v>66</v>
       </c>
@@ -2293,8 +2596,11 @@
         <v>66</v>
       </c>
       <c r="C98" s="66"/>
-    </row>
-    <row r="99" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D98" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A99" s="71" t="s">
         <v>67</v>
       </c>
@@ -2302,8 +2608,11 @@
         <v>67</v>
       </c>
       <c r="C99" s="67"/>
-    </row>
-    <row r="100" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D99" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A100" s="71" t="s">
         <v>68</v>
       </c>
@@ -2313,8 +2622,11 @@
       <c r="C100" s="68">
         <v>71000</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D100" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A101" s="71" t="s">
         <v>69</v>
       </c>
@@ -2322,8 +2634,11 @@
         <v>69</v>
       </c>
       <c r="C101" s="69"/>
-    </row>
-    <row r="102" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D101" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A102" s="71" t="s">
         <v>70</v>
       </c>
@@ -2333,8 +2648,11 @@
       <c r="C102" s="66">
         <v>64000</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D102" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A103" s="71" t="s">
         <v>71</v>
       </c>
@@ -2342,8 +2660,11 @@
         <v>71</v>
       </c>
       <c r="C103" s="66"/>
-    </row>
-    <row r="104" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D103" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A104" s="71" t="s">
         <v>72</v>
       </c>
@@ -2351,8 +2672,11 @@
         <v>72</v>
       </c>
       <c r="C104" s="66"/>
-    </row>
-    <row r="105" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D104" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A105" s="71" t="s">
         <v>73</v>
       </c>
@@ -2360,8 +2684,11 @@
         <v>73</v>
       </c>
       <c r="C105" s="67"/>
-    </row>
-    <row r="106" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D105" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A106" s="71" t="s">
         <v>74</v>
       </c>
@@ -2371,8 +2698,11 @@
       <c r="C106" s="68">
         <v>71000</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D106" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A107" s="71" t="s">
         <v>75</v>
       </c>
@@ -2380,8 +2710,11 @@
         <v>75</v>
       </c>
       <c r="C107" s="68"/>
-    </row>
-    <row r="108" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D107" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A108" s="71" t="s">
         <v>76</v>
       </c>
@@ -2391,8 +2724,11 @@
       <c r="C108" s="70">
         <v>68203</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D108" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A109" s="71" t="s">
         <v>77</v>
       </c>
@@ -2400,8 +2736,11 @@
         <v>77</v>
       </c>
       <c r="C109" s="12"/>
-    </row>
-    <row r="110" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D109" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A110" s="71" t="s">
         <v>78</v>
       </c>
@@ -2411,8 +2750,11 @@
       <c r="C110" s="68">
         <v>71000</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D110" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A111" s="71" t="s">
         <v>79</v>
       </c>
@@ -2420,8 +2762,11 @@
         <v>79</v>
       </c>
       <c r="C111" s="37"/>
-    </row>
-    <row r="112" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D111" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A112" s="71" t="s">
         <v>80</v>
       </c>
@@ -2429,8 +2774,11 @@
         <v>80</v>
       </c>
       <c r="C112" s="37"/>
-    </row>
-    <row r="113" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D112" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A113" s="71" t="s">
         <v>81</v>
       </c>
@@ -2438,8 +2786,11 @@
         <v>81</v>
       </c>
       <c r="C113" s="37"/>
-    </row>
-    <row r="114" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D113" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A114" s="71" t="s">
         <v>82</v>
       </c>
@@ -2447,8 +2798,11 @@
         <v>82</v>
       </c>
       <c r="C114" s="37"/>
-    </row>
-    <row r="115" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D114" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A115" s="71" t="s">
         <v>83</v>
       </c>
@@ -2458,8 +2812,11 @@
       <c r="C115" s="41" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D115" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A116" s="71" t="s">
         <v>84</v>
       </c>
@@ -2469,8 +2826,11 @@
       <c r="C116" s="66">
         <v>71000</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D116" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A117" s="71" t="s">
         <v>85</v>
       </c>
@@ -2478,8 +2838,11 @@
         <v>85</v>
       </c>
       <c r="C117" s="34"/>
-    </row>
-    <row r="118" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D117" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A118" s="71" t="s">
         <v>86</v>
       </c>
@@ -2487,8 +2850,11 @@
         <v>86</v>
       </c>
       <c r="C118" s="34"/>
-    </row>
-    <row r="119" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D118" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A119" s="71" t="s">
         <v>87</v>
       </c>
@@ -2496,8 +2862,11 @@
         <v>87</v>
       </c>
       <c r="C119" s="34"/>
-    </row>
-    <row r="120" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D119" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A120" s="71" t="s">
         <v>88</v>
       </c>
@@ -2505,8 +2874,11 @@
         <v>88</v>
       </c>
       <c r="C120" s="35"/>
-    </row>
-    <row r="121" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D120" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A121" s="71" t="s">
         <v>89</v>
       </c>
@@ -2516,8 +2888,11 @@
       <c r="C121" s="41">
         <v>55560</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D121" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A122" s="71" t="s">
         <v>90</v>
       </c>
@@ -2527,8 +2902,11 @@
       <c r="C122" s="68">
         <v>71000</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D122" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A123" s="71" t="s">
         <v>91</v>
       </c>
@@ -2536,8 +2914,11 @@
         <v>91</v>
       </c>
       <c r="C123" s="37"/>
-    </row>
-    <row r="124" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D123" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A124" s="71" t="s">
         <v>92</v>
       </c>
@@ -2545,8 +2926,11 @@
         <v>92</v>
       </c>
       <c r="C124" s="37"/>
-    </row>
-    <row r="125" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D124" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A125" s="71" t="s">
         <v>93</v>
       </c>
@@ -2556,8 +2940,11 @@
       <c r="C125" s="52" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D125" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A126" s="73" t="s">
         <v>94</v>
       </c>
@@ -2565,8 +2952,11 @@
         <v>94</v>
       </c>
       <c r="C126" s="40"/>
-    </row>
-    <row r="127" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D126" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A127" s="71" t="s">
         <v>95</v>
       </c>
@@ -2576,8 +2966,11 @@
       <c r="C127" s="52">
         <v>55560</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D127" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A128" s="71" t="s">
         <v>96</v>
       </c>
@@ -2587,8 +2980,11 @@
       <c r="C128" s="52" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D128" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A129" s="71" t="s">
         <v>97</v>
       </c>
@@ -2596,8 +2992,11 @@
         <v>97</v>
       </c>
       <c r="C129" s="37"/>
-    </row>
-    <row r="130" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D129" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A130" s="71" t="s">
         <v>98</v>
       </c>
@@ -2605,8 +3004,11 @@
         <v>98</v>
       </c>
       <c r="C130" s="37"/>
-    </row>
-    <row r="131" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D130" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A131" s="71" t="s">
         <v>99</v>
       </c>
@@ -2614,8 +3016,11 @@
         <v>99</v>
       </c>
       <c r="C131" s="40"/>
-    </row>
-    <row r="132" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D131" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A132" s="71" t="s">
         <v>100</v>
       </c>
@@ -2625,8 +3030,11 @@
       <c r="C132" s="68">
         <v>71000</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D132" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A133" s="71" t="s">
         <v>101</v>
       </c>
@@ -2636,8 +3044,11 @@
       <c r="C133" s="52" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D133" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A134" s="71" t="s">
         <v>102</v>
       </c>
@@ -2645,8 +3056,11 @@
         <v>102</v>
       </c>
       <c r="C134" s="37"/>
-    </row>
-    <row r="135" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D134" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A135" s="71" t="s">
         <v>103</v>
       </c>
@@ -2654,8 +3068,11 @@
         <v>103</v>
       </c>
       <c r="C135" s="37"/>
-    </row>
-    <row r="136" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D135" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A136" s="71" t="s">
         <v>104</v>
       </c>
@@ -2663,8 +3080,11 @@
         <v>104</v>
       </c>
       <c r="C136" s="37"/>
-    </row>
-    <row r="137" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D136" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A137" s="71" t="s">
         <v>105</v>
       </c>
@@ -2672,8 +3092,11 @@
         <v>105</v>
       </c>
       <c r="C137" s="37"/>
-    </row>
-    <row r="138" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D137" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A138" s="71" t="s">
         <v>106</v>
       </c>
@@ -2681,8 +3104,11 @@
         <v>106</v>
       </c>
       <c r="C138" s="37"/>
-    </row>
-    <row r="139" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D138" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A139" s="71" t="s">
         <v>107</v>
       </c>
@@ -2690,8 +3116,11 @@
         <v>107</v>
       </c>
       <c r="C139" s="37"/>
-    </row>
-    <row r="140" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D139" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A140" s="71" t="s">
         <v>108</v>
       </c>
@@ -2699,8 +3128,11 @@
         <v>108</v>
       </c>
       <c r="C140" s="40"/>
-    </row>
-    <row r="141" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D140" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A141" s="71" t="s">
         <v>109</v>
       </c>
@@ -2710,8 +3142,11 @@
       <c r="C141" s="68">
         <v>55560</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D141" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A142" s="71" t="s">
         <v>110</v>
       </c>
@@ -2719,8 +3154,11 @@
         <v>110</v>
       </c>
       <c r="C142" s="37"/>
-    </row>
-    <row r="143" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D142" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A143" s="71" t="s">
         <v>111</v>
       </c>
@@ -2728,8 +3166,11 @@
         <v>111</v>
       </c>
       <c r="C143" s="37"/>
-    </row>
-    <row r="144" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D143" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A144" s="71" t="s">
         <v>112</v>
       </c>
@@ -2737,8 +3178,11 @@
         <v>112</v>
       </c>
       <c r="C144" s="37"/>
-    </row>
-    <row r="145" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D144" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A145" s="71" t="s">
         <v>113</v>
       </c>
@@ -2746,8 +3190,11 @@
         <v>113</v>
       </c>
       <c r="C145" s="37"/>
-    </row>
-    <row r="146" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D145" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A146" s="71" t="s">
         <v>114</v>
       </c>
@@ -2755,8 +3202,11 @@
         <v>114</v>
       </c>
       <c r="C146" s="37"/>
-    </row>
-    <row r="147" spans="1:3" ht="18" x14ac:dyDescent="0.45">
+      <c r="D146" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" ht="18" x14ac:dyDescent="0.45">
       <c r="A147" s="71" t="s">
         <v>115</v>
       </c>
@@ -2764,6 +3214,9 @@
         <v>115</v>
       </c>
       <c r="C147" s="40"/>
+      <c r="D147" t="s">
+        <v>179</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>